<commit_message>
NSTA-136 Added checking of quote statuses though different state. Added code to upload b2b prices. Creating contracts with 'Customer switch' type. See further how to handle creation of more contracts with the same address and ean. Remarks. On uat*, B2B TC1 contract is not active, on devint02 it is (probably configuration is different)
</commit_message>
<xml_diff>
--- a/src/test/resources/data/contract_b2b/address_b2b/adress_b2B.XLSX
+++ b/src/test/resources/data/contract_b2b/address_b2b/adress_b2B.XLSX
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="19126"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100800_{242DE730-079B-4482-B61C-C634325406E2}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="60" windowWidth="17100" windowHeight="6030" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18375" windowHeight="6285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ELEC" sheetId="1" r:id="rId1"/>
     <sheet name="GAS" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A127:K144"/>
 </workbook>
 </file>
 
@@ -1818,7 +1820,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1860,6 +1862,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1908,7 +1913,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1941,9 +1946,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1976,6 +1998,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2151,7 +2190,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B230"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4006,7 +4045,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4588,7 +4627,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>